<commit_message>
Update R2450_51_52_CLIENTES POR PRODUCTO_V0.5 -- R2450 - R2451 - R2452.xlsx
</commit_message>
<xml_diff>
--- a/Documentación/OPERATIVOS/R2450_51_52_CLIENTES POR PRODUCTO_V0.5 -- R2450 - R2451 - R2452.xlsx
+++ b/Documentación/OPERATIVOS/R2450_51_52_CLIENTES POR PRODUCTO_V0.5 -- R2450 - R2451 - R2452.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edgar.rojas\Documents\1408\formatos PMO\planes de trabajo\Bajaware\Layouts Bw confidencial\Layouts\OPERATIVOS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/808f7a51c3ffcfac/Documentos/GitHub/ION_reportesregulatorios/Documentación/OPERATIVOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF6F493-7973-43F2-95F1-4F2D849C67BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{6CF6F493-7973-43F2-95F1-4F2D849C67BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B49474EC-8676-4F43-A210-92056D5EA468}"/>
   <bookViews>
-    <workbookView xWindow="2268" yWindow="504" windowWidth="15420" windowHeight="16512" xr2:uid="{DFB8C20A-8D75-254E-939C-21ACB005D1C5}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DFB8C20A-8D75-254E-939C-21ACB005D1C5}"/>
   </bookViews>
   <sheets>
     <sheet name="CLIENTES POR PRODUCTO" sheetId="1" r:id="rId1"/>
@@ -485,9 +485,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -525,7 +525,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -631,7 +631,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -773,7 +773,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -782,19 +782,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A0AB60D-8446-DE43-84C8-ABB6B1BBEC37}">
   <dimension ref="A1:T19"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
-    <col min="4" max="4" width="22.5" customWidth="1"/>
-    <col min="5" max="5" width="14.375" customWidth="1"/>
-    <col min="9" max="9" width="58.125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="90.625" customWidth="1"/>
+    <col min="1" max="1" width="45.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.8984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.8984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.59765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.19921875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="59.19921875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="28.8984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="90.59765625" customWidth="1"/>
+    <col min="13" max="13" width="22.796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.8984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24.19921875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1"/>
     </row>
-    <row r="2" spans="1:20" ht="31.15">
+    <row r="2" spans="1:20" ht="31.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -890,7 +901,7 @@
       <c r="S5" s="5"/>
       <c r="T5" s="4"/>
     </row>
-    <row r="6" spans="1:20" ht="31.15">
+    <row r="6" spans="1:20" ht="31.2">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -931,7 +942,7 @@
       <c r="S6" s="5"/>
       <c r="T6" s="4"/>
     </row>
-    <row r="7" spans="1:20" ht="124.9">
+    <row r="7" spans="1:20" ht="124.8">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -972,7 +983,7 @@
       <c r="S7" s="5"/>
       <c r="T7" s="4"/>
     </row>
-    <row r="8" spans="1:20" ht="46.9">
+    <row r="8" spans="1:20" ht="46.8">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -1087,7 +1098,7 @@
       <c r="R10" s="5"/>
       <c r="S10" s="5"/>
     </row>
-    <row r="11" spans="1:20" ht="31.15">
+    <row r="11" spans="1:20" ht="31.2">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -1252,6 +1263,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="cf35dce2-b600-471d-a6b0-9e8301b7851b">
@@ -1260,15 +1280,6 @@
     <TaxCatchAll xmlns="3de82841-ffbb-418b-a888-39c303bacd30" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1473,13 +1484,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6343FABE-295D-4E5F-B1B7-C6657EEDE556}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{59D4C7A6-80A4-4B27-A218-B1B1074CD177}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{59D4C7A6-80A4-4B27-A218-B1B1074CD177}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6343FABE-295D-4E5F-B1B7-C6657EEDE556}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="cf35dce2-b600-471d-a6b0-9e8301b7851b"/>
+    <ds:schemaRef ds:uri="3de82841-ffbb-418b-a888-39c303bacd30"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27DE4CD4-2746-4815-B8C4-716D13074C4F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27DE4CD4-2746-4815-B8C4-716D13074C4F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="cf35dce2-b600-471d-a6b0-9e8301b7851b"/>
+    <ds:schemaRef ds:uri="3de82841-ffbb-418b-a888-39c303bacd30"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>